<commit_message>
feat: upgrade all 120 challenges to realistic engineering defects with 100% test validation
</commit_message>
<xml_diff>
--- a/testing/BUG_REPORTS.xlsx
+++ b/testing/BUG_REPORTS.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -458,8 +458,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="83" customWidth="1" min="8" max="8"/>
-    <col width="108" customWidth="1" min="9" max="9"/>
+    <col width="93" customWidth="1" min="8" max="8"/>
+    <col width="112" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -694,6 +694,147 @@
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Linked User profile interests, strengths, and weaknesses directly to Career Engine ML service</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BUG-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Arbitrary / Fake emails accepted during signup and login</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Absence of domain legitimacy regex in frontend and backend email validators</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Added strict email validator in frontend utils and Django backend rejecting invalid domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BUG-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>New user initialized with hardcoded 5-day streak and fake bio</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Hardcoded mock notification in App.jsx and mock profile fields in views.py</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Cleared default notifications and initialized new users with 0 streak, 0 solved, empty badges</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BUG-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>OTP verification bypassed with arbitrary 6-digit number</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>views.py contained fallback 'elif len(otp) == 6: otp_valid = True' bypassing verification</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Removed mock bypass, hooked real Gmail SMTP credentials, enforced cache verification and single-use eviction</t>
         </is>
       </c>
     </row>

</xml_diff>